<commit_message>
v154: Template-based Excel export with ExcelJS + diacritics-insensitive matching
- Replace programmatic SheetJS export with user's exact V1/V2 Excel templates
- Add ExcelJS CDN lazy-loader for template manipulation (preserves all formatting)
- Embed templates as base64 in js/template-data.js for offline PWA support
- Diacritics-insensitive operation matching (_normOp): "Curatare" matches "Curățare"
- Operations not in template auto-added as new columns (J, K, ...)
- V1 (Chimicale): maps stock products to fixed template columns C-J
- V2 (Servicii): reads R10 headers, matches checked operations, places checkmarks
- Dynamic row insertion/deletion via spliceRows for variable intervention counts
- Formula auto-update (COUNT, SUM, IFERROR) to match actual data range
- Legacy SheetJS functions kept as fallback (_legacy suffix)
- Bump SW to v154, APP_VERSION to 154

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/v1.xlsx
+++ b/templates/v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ceorn\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{689E0F76-2832-439A-AFD1-2DD95C2F92B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{544784F2-8C2D-4803-A72B-ED16ADEA5E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,11 +40,6 @@
 0721.137.178</t>
   </si>
   <si>
-    <t>J40/18144/2007
-CUI: RO22479681
-RO77RNCB0074092331280001</t>
-  </si>
-  <si>
     <t>RAPORT INTERVENȚII — CHIMICALE PISCINĂ</t>
   </si>
   <si>
@@ -52,10 +47,6 @@
 intervenție</t>
   </si>
   <si>
-    <t>Cant.
-(l/kg)</t>
-  </si>
-  <si>
     <t>CHIMICALE FOLOSITE</t>
   </si>
   <si>
@@ -101,13 +92,37 @@
   </si>
   <si>
     <t>S.C. Aquatis Engineering S.R.L.</t>
+  </si>
+  <si>
+    <t>Client</t>
+  </si>
+  <si>
+    <t>Nr. Document</t>
+  </si>
+  <si>
+    <t>Data emiterii</t>
+  </si>
+  <si>
+    <t>Toate prețurile sunt exprimate în RON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                                                     J40/18144/2007
+                                                                  CUI: RO22479681
+                                            RO77RNCB0074092331280001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cant.
+</t>
+  </si>
+  <si>
+    <t>Perioada raportata</t>
   </si>
   <si>
     <r>
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FF0D2D5A"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
@@ -117,7 +132,7 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color rgb="FF0D2D5A"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
@@ -128,27 +143,12 @@
       <rPr>
         <b/>
         <sz val="10"/>
-        <color rgb="FF0D2D5A"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>Str. Eufrosina Popescu 50, Sector 3</t>
     </r>
-  </si>
-  <si>
-    <t>Client</t>
-  </si>
-  <si>
-    <t>Luna / Perioada</t>
-  </si>
-  <si>
-    <t>Nr. Document</t>
-  </si>
-  <si>
-    <t>Data emiterii</t>
-  </si>
-  <si>
-    <t>Toate prețurile sunt exprimate în RON</t>
   </si>
 </sst>
 </file>
@@ -158,7 +158,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -169,11 +169,6 @@
     <font>
       <sz val="9"/>
       <color rgb="FF0D2D5A"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="8.5"/>
-      <color rgb="FF2A5070"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -213,26 +208,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <i/>
-      <sz val="7.5"/>
-      <color rgb="FF4A7A99"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF0D2D5A"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF0D2D5A"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF0D2D5A"/>
@@ -254,11 +229,48 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8.5"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <i/>
       <sz val="7.5"/>
-      <color rgb="FF4A7A99"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="7.5"/>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="13">
@@ -271,11 +283,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0D2D5A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF4DB8E8"/>
       </patternFill>
     </fill>
     <fill>
@@ -327,6 +334,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="39">
     <border>
@@ -846,139 +859,142 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="4" fontId="1" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="8" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="7" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="6" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="4" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="4" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="11" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="11" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="4" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="4" fillId="12" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="7" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="5" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="5" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="5" fillId="10" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="3" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="5" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="12" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -987,6 +1003,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFCE7D10"/>
       <color rgb="FF1D507F"/>
     </mruColors>
   </colors>
@@ -1303,177 +1320,177 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="3.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="7"/>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-    </row>
-    <row r="2" spans="1:11" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="56" t="s">
+      <c r="A1" s="27"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+    </row>
+    <row r="2" spans="1:11" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="46" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="45"/>
+    </row>
+    <row r="3" spans="1:11" ht="3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="54"/>
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
+    </row>
+    <row r="4" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="40" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="42"/>
+    </row>
+    <row r="5" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="57"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="52" t="s">
-        <v>1</v>
-      </c>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-      <c r="K2" s="54"/>
-    </row>
-    <row r="3" spans="1:11" ht="3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="10"/>
-    </row>
-    <row r="4" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="33" t="s">
+      <c r="K5" s="24"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="43"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="33"/>
+    </row>
+    <row r="7" spans="1:11" ht="3.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="34"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="35"/>
+    </row>
+    <row r="8" spans="1:11" ht="26.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="35"/>
-    </row>
-    <row r="5" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="44" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="44" t="s">
+      <c r="B8" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="H5" s="43"/>
-      <c r="I5" s="43"/>
-      <c r="J5" s="44" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" s="45"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="13"/>
-    </row>
-    <row r="7" spans="1:11" ht="3.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="14"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="10"/>
-    </row>
-    <row r="8" spans="1:11" ht="26.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="23" t="s">
+      <c r="C8" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="23" t="s">
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="38"/>
+      <c r="I8" s="38"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="25" t="s">
+    </row>
+    <row r="9" spans="1:11" ht="32.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="36"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="27"/>
-      <c r="K8" s="23" t="s">
+      <c r="D9" s="52" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="32.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="24"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="48" t="s">
+      <c r="E9" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="F9" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="46" t="s">
+      <c r="G9" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="46" t="s">
+      <c r="H9" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="46" t="s">
+      <c r="I9" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="46" t="s">
+      <c r="J9" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="46" t="s">
-        <v>13</v>
-      </c>
-      <c r="J9" s="47" t="s">
-        <v>14</v>
-      </c>
-      <c r="K9" s="24"/>
+      <c r="K9" s="36"/>
     </row>
     <row r="10" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="28"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
-      <c r="K10" s="30"/>
+      <c r="A10" s="10"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="12"/>
     </row>
     <row r="11" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="58"/>
+      <c r="A11" s="16"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -1483,10 +1500,10 @@
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
-      <c r="K11" s="17"/>
+      <c r="K11" s="7"/>
     </row>
     <row r="12" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="15"/>
+      <c r="A12" s="5"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -1496,10 +1513,10 @@
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
-      <c r="K12" s="16"/>
+      <c r="K12" s="6"/>
     </row>
     <row r="13" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="58"/>
+      <c r="A13" s="16"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -1509,10 +1526,10 @@
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
-      <c r="K13" s="17"/>
+      <c r="K13" s="7"/>
     </row>
     <row r="14" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="15"/>
+      <c r="A14" s="5"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -1522,10 +1539,10 @@
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
-      <c r="K14" s="16"/>
+      <c r="K14" s="6"/>
     </row>
     <row r="15" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="58"/>
+      <c r="A15" s="16"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -1535,10 +1552,10 @@
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
-      <c r="K15" s="17"/>
+      <c r="K15" s="7"/>
     </row>
     <row r="16" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
+      <c r="A16" s="5"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -1548,10 +1565,10 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
-      <c r="K16" s="16"/>
+      <c r="K16" s="6"/>
     </row>
     <row r="17" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="58"/>
+      <c r="A17" s="16"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -1561,10 +1578,10 @@
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
-      <c r="K17" s="17"/>
+      <c r="K17" s="7"/>
     </row>
     <row r="18" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15"/>
+      <c r="A18" s="5"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -1574,63 +1591,63 @@
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
-      <c r="K18" s="16"/>
+      <c r="K18" s="6"/>
     </row>
     <row r="19" spans="1:11" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="59"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="31"/>
-      <c r="H19" s="31"/>
-      <c r="I19" s="31"/>
-      <c r="J19" s="31"/>
-      <c r="K19" s="32"/>
+      <c r="A19" s="17"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="14"/>
     </row>
     <row r="20" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="B20" s="37"/>
-      <c r="C20" s="38">
+      <c r="A20" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="58"/>
+      <c r="C20" s="59">
         <f t="shared" ref="C20:J20" si="0">SUM(C10:C19)</f>
         <v>0</v>
       </c>
-      <c r="D20" s="38">
+      <c r="D20" s="59">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E20" s="38">
+      <c r="E20" s="59">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F20" s="38">
+      <c r="F20" s="59">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G20" s="38">
+      <c r="G20" s="59">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="38">
+      <c r="H20" s="59">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I20" s="38">
+      <c r="I20" s="59">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J20" s="38">
+      <c r="J20" s="59">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K20" s="39"/>
+      <c r="K20" s="60"/>
     </row>
     <row r="21" spans="1:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="18" t="s">
-        <v>16</v>
+      <c r="A21" s="8" t="s">
+        <v>14</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="4">
@@ -1657,77 +1674,69 @@
       <c r="J21" s="4">
         <v>180</v>
       </c>
-      <c r="K21" s="19"/>
+      <c r="K21" s="9"/>
     </row>
     <row r="22" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="49" t="s">
-        <v>17</v>
-      </c>
-      <c r="B22" s="50"/>
-      <c r="C22" s="51">
+      <c r="A22" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="19"/>
+      <c r="C22" s="20">
         <f t="shared" ref="C22:J22" si="1">C20*C21</f>
         <v>0</v>
       </c>
-      <c r="D22" s="51">
+      <c r="D22" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E22" s="51">
+      <c r="E22" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F22" s="51">
+      <c r="F22" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G22" s="51">
+      <c r="G22" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H22" s="51">
+      <c r="H22" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I22" s="51">
+      <c r="I22" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J22" s="51">
+      <c r="J22" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K22" s="40">
+      <c r="K22" s="15">
         <f>SUM(C22,D22,E22,F22,G22,H22,I22,J22)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="41" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="22"/>
+    <row r="23" spans="1:11" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="48"/>
+      <c r="C23" s="48"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
+      <c r="H23" s="49" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" s="48"/>
+      <c r="J23" s="48"/>
+      <c r="K23" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="H2:K2"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="A23:G23"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="B8:B9"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="H23:K23"/>
     <mergeCell ref="E2:G2"/>
@@ -1741,6 +1750,14 @@
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="C8:J8"/>
     <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="B8:B9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>